<commit_message>
Atualiza base de dados (dPartidas, dTimes, fDespesas, fFacial, fIngressos)
Regenera data.js: 82 partidas, 1566 bordero rows, 3983 ingressos rows
KPIs: público total 1.610.092 · ticket médio R$ 31,41 · % sócios 62,6%

https://claude.ai/code/session_01Bb3ciycnMnk9Z7WYwsqMvC
</commit_message>
<xml_diff>
--- a/dPartidas.xlsx
+++ b/dPartidas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="EstaPastaDeTrabalho" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://safbotafogo-my.sharepoint.com/personal/pedro_arruda_safbfr_com_br/Documents/BI/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://safbotafogo-my.sharepoint.com/personal/pedro_arruda_safbfr_com_br/Documents/Área de Trabalho/dash-ticket/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="296" documentId="8_{E25D5179-CBFE-42C3-9E8D-799BA19C3FB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A72B6E0D-2D08-47BD-AD4B-0FC36731CE92}"/>
+  <xr:revisionPtr revIDLastSave="477" documentId="8_{E25D5179-CBFE-42C3-9E8D-799BA19C3FB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15D5C576-7611-44B6-AFD0-EE56B32D2144}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E1B40A1D-D5F1-4DC5-B00D-B969B491F639}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E1B40A1D-D5F1-4DC5-B00D-B969B491F639}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha3" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="158">
   <si>
     <t>ID_PARTIDA</t>
   </si>
@@ -423,6 +423,96 @@
   </si>
   <si>
     <t>2025.10.15-CAMBR2-28</t>
+  </si>
+  <si>
+    <t>3° Fase</t>
+  </si>
+  <si>
+    <t>Quartas</t>
+  </si>
+  <si>
+    <t>SEMIS - TR</t>
+  </si>
+  <si>
+    <t>FINAL - TR</t>
+  </si>
+  <si>
+    <t>2025.10.26-CAMBR2-30</t>
+  </si>
+  <si>
+    <t>2025.11.05-CAMBR2-32</t>
+  </si>
+  <si>
+    <t>2025.11.18-CAMBR2-34</t>
+  </si>
+  <si>
+    <t>2025.11.22-CAMBR2-35</t>
+  </si>
+  <si>
+    <t>2025.12.07-CAMBR2-38</t>
+  </si>
+  <si>
+    <t>2026.01.21-CAMCA4-3</t>
+  </si>
+  <si>
+    <t>2026.01.24-CAMCA4-4</t>
+  </si>
+  <si>
+    <t>2026.01.29-CAMBR2-1</t>
+  </si>
+  <si>
+    <t>2026.02.01-CAMCA4-5</t>
+  </si>
+  <si>
+    <t>2026.02.15-CAMCA4-Quartas</t>
+  </si>
+  <si>
+    <t>2026.02.25-CAMLI5-2° FASE</t>
+  </si>
+  <si>
+    <t>2026.02.28-CAMCA4-SEMIS - TR</t>
+  </si>
+  <si>
+    <t>2026.03.07-CAMCA4-FINAL - TR</t>
+  </si>
+  <si>
+    <t>2026.03.10-CAMLI5-3° Fase</t>
+  </si>
+  <si>
+    <t>2026.03.14-CAMBR2-6</t>
+  </si>
+  <si>
+    <t>2026.04.01-CAMBR2-9</t>
+  </si>
+  <si>
+    <t>7SABRSP</t>
+  </si>
+  <si>
+    <t>10GRBRRS</t>
+  </si>
+  <si>
+    <t>13SPBRPE</t>
+  </si>
+  <si>
+    <t>93BAECGU</t>
+  </si>
+  <si>
+    <t>123NABOPO</t>
+  </si>
+  <si>
+    <t>CAMSU6</t>
+  </si>
+  <si>
+    <t>12COBRPR</t>
+  </si>
+  <si>
+    <t>115CAVECA</t>
+  </si>
+  <si>
+    <t>2026.04.09-CAMSU6-FG</t>
+  </si>
+  <si>
+    <t>2026.04.12-CAMBR2-11</t>
   </si>
 </sst>
 </file>
@@ -452,12 +542,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -472,7 +574,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -480,6 +582,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -816,13 +928,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2921BBCD-6E27-463C-B492-0BF065778598}">
   <sheetPr codeName="Planilha1"/>
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G83"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.81640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.90625" style="4" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.81640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.81640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -840,7 +953,7 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -978,7 +1091,7 @@
       <c r="D7" s="2">
         <v>45350</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="4" t="s">
         <v>67</v>
       </c>
       <c r="F7" t="s">
@@ -1001,7 +1114,7 @@
       <c r="D8" s="2">
         <v>45357</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="4" t="s">
         <v>68</v>
       </c>
       <c r="F8" t="s">
@@ -1070,7 +1183,7 @@
       <c r="D11" s="2">
         <v>45385</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="4" t="s">
         <v>69</v>
       </c>
       <c r="F11" t="s">
@@ -1139,7 +1252,7 @@
       <c r="D14" s="2">
         <v>45406</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="4" t="s">
         <v>69</v>
       </c>
       <c r="F14" t="s">
@@ -1162,7 +1275,7 @@
       <c r="D15" s="2">
         <v>45414</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="4" t="s">
         <v>68</v>
       </c>
       <c r="F15" t="s">
@@ -1208,7 +1321,7 @@
       <c r="D17" s="2">
         <v>45420</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="4" t="s">
         <v>69</v>
       </c>
       <c r="F17" t="s">
@@ -1392,7 +1505,7 @@
       <c r="D25" s="2">
         <v>45503</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" s="4" t="s">
         <v>70</v>
       </c>
       <c r="F25" t="s">
@@ -1406,16 +1519,13 @@
       <c r="A26" t="s">
         <v>79</v>
       </c>
-      <c r="B26" t="s">
-        <v>73</v>
-      </c>
       <c r="C26" t="s">
         <v>27</v>
       </c>
       <c r="D26" s="2">
         <v>45518</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E26" s="4" t="s">
         <v>70</v>
       </c>
       <c r="F26" t="s">
@@ -1507,7 +1617,7 @@
       <c r="D30" s="2">
         <v>45553</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E30" s="4" t="s">
         <v>71</v>
       </c>
       <c r="F30" t="s">
@@ -1530,7 +1640,7 @@
       <c r="D31" s="2">
         <v>45560</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E31" s="4" t="s">
         <v>71</v>
       </c>
       <c r="F31" t="s">
@@ -1553,7 +1663,7 @@
       <c r="D32" s="2">
         <v>45583</v>
       </c>
-      <c r="E32">
+      <c r="E32" s="4">
         <v>30</v>
       </c>
       <c r="F32" t="s">
@@ -1576,7 +1686,7 @@
       <c r="D33" s="2">
         <v>45588</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E33" s="4" t="s">
         <v>72</v>
       </c>
       <c r="F33" t="s">
@@ -1599,7 +1709,7 @@
       <c r="D34" s="2">
         <v>45595</v>
       </c>
-      <c r="E34" t="s">
+      <c r="E34" s="4" t="s">
         <v>72</v>
       </c>
       <c r="F34" t="s">
@@ -1714,7 +1824,7 @@
       <c r="D39" s="2">
         <v>45668</v>
       </c>
-      <c r="E39">
+      <c r="E39" s="4">
         <v>1</v>
       </c>
       <c r="F39" t="s">
@@ -1737,7 +1847,7 @@
       <c r="D40" s="2">
         <v>45671</v>
       </c>
-      <c r="E40">
+      <c r="E40" s="4">
         <v>2</v>
       </c>
       <c r="F40" t="s">
@@ -1760,7 +1870,7 @@
       <c r="D41" s="2">
         <v>45679</v>
       </c>
-      <c r="E41">
+      <c r="E41" s="4">
         <v>4</v>
       </c>
       <c r="F41" t="s">
@@ -1783,7 +1893,7 @@
       <c r="D42" s="2">
         <v>45683</v>
       </c>
-      <c r="E42">
+      <c r="E42" s="4">
         <v>5</v>
       </c>
       <c r="F42" t="s">
@@ -1806,7 +1916,7 @@
       <c r="D43" s="2">
         <v>45686</v>
       </c>
-      <c r="E43">
+      <c r="E43" s="4">
         <v>6</v>
       </c>
       <c r="F43" t="s">
@@ -1817,7 +1927,7 @@
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A44" s="5" t="s">
+      <c r="A44" t="s">
         <v>107</v>
       </c>
       <c r="B44" t="s">
@@ -1829,7 +1939,7 @@
       <c r="D44" s="2">
         <v>45715</v>
       </c>
-      <c r="E44" t="s">
+      <c r="E44" s="4" t="s">
         <v>104</v>
       </c>
       <c r="F44" t="s">
@@ -1840,7 +1950,7 @@
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A45" s="5" t="s">
+      <c r="A45" t="s">
         <v>96</v>
       </c>
       <c r="B45" t="s">
@@ -1852,7 +1962,7 @@
       <c r="D45" s="2">
         <v>45752</v>
       </c>
-      <c r="E45">
+      <c r="E45" s="4">
         <v>2</v>
       </c>
       <c r="F45" t="s">
@@ -1863,7 +1973,7 @@
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A46" s="5" t="s">
+      <c r="A46" t="s">
         <v>97</v>
       </c>
       <c r="B46" t="s">
@@ -1875,7 +1985,7 @@
       <c r="D46" s="2">
         <v>45755</v>
       </c>
-      <c r="E46">
+      <c r="E46" s="4">
         <v>2</v>
       </c>
       <c r="F46" t="s">
@@ -1886,7 +1996,7 @@
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A47" s="5" t="s">
+      <c r="A47" t="s">
         <v>98</v>
       </c>
       <c r="B47" t="s">
@@ -1898,7 +2008,7 @@
       <c r="D47" s="2">
         <v>45763</v>
       </c>
-      <c r="E47">
+      <c r="E47" s="4">
         <v>4</v>
       </c>
       <c r="F47" t="s">
@@ -1909,7 +2019,7 @@
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A48" s="5" t="s">
+      <c r="A48" t="s">
         <v>99</v>
       </c>
       <c r="B48" t="s">
@@ -1921,7 +2031,7 @@
       <c r="D48" s="2">
         <v>45773</v>
       </c>
-      <c r="E48">
+      <c r="E48" s="4">
         <v>6</v>
       </c>
       <c r="F48" t="s">
@@ -1932,7 +2042,7 @@
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A49" s="5" t="s">
+      <c r="A49" t="s">
         <v>100</v>
       </c>
       <c r="B49" t="s">
@@ -1944,7 +2054,7 @@
       <c r="D49" s="2">
         <v>45777</v>
       </c>
-      <c r="E49" t="s">
+      <c r="E49" s="4" t="s">
         <v>68</v>
       </c>
       <c r="F49" t="s">
@@ -1955,7 +2065,7 @@
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A50" s="5" t="s">
+      <c r="A50" t="s">
         <v>106</v>
       </c>
       <c r="B50" t="s">
@@ -1967,7 +2077,7 @@
       <c r="D50" s="2">
         <v>45788</v>
       </c>
-      <c r="E50">
+      <c r="E50" s="4">
         <v>8</v>
       </c>
       <c r="F50" t="s">
@@ -1978,7 +2088,7 @@
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A51" s="5" t="s">
+      <c r="A51" t="s">
         <v>109</v>
       </c>
       <c r="B51" t="s">
@@ -1990,7 +2100,7 @@
       <c r="D51" s="2">
         <v>45791</v>
       </c>
-      <c r="E51">
+      <c r="E51" s="4">
         <v>5</v>
       </c>
       <c r="F51" t="s">
@@ -2001,7 +2111,7 @@
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A52" s="5" t="s">
+      <c r="A52" t="s">
         <v>111</v>
       </c>
       <c r="B52" t="s">
@@ -2013,7 +2123,7 @@
       <c r="D52" s="2">
         <v>45804</v>
       </c>
-      <c r="E52">
+      <c r="E52" s="4">
         <v>6</v>
       </c>
       <c r="F52" t="s">
@@ -2024,7 +2134,7 @@
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A53" s="5" t="s">
+      <c r="A53" t="s">
         <v>114</v>
       </c>
       <c r="B53" t="s">
@@ -2036,7 +2146,7 @@
       <c r="D53" s="2">
         <v>45812</v>
       </c>
-      <c r="E53">
+      <c r="E53" s="4">
         <v>10</v>
       </c>
       <c r="F53" t="s">
@@ -2047,7 +2157,7 @@
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A54" s="5" t="s">
+      <c r="A54" t="s">
         <v>115</v>
       </c>
       <c r="B54" t="s">
@@ -2059,7 +2169,7 @@
       <c r="D54" s="2">
         <v>45854</v>
       </c>
-      <c r="E54">
+      <c r="E54" s="4">
         <v>14</v>
       </c>
       <c r="F54" t="s">
@@ -2070,7 +2180,7 @@
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A55" s="5" t="s">
+      <c r="A55" t="s">
         <v>116</v>
       </c>
       <c r="B55" t="s">
@@ -2082,7 +2192,7 @@
       <c r="D55" s="2">
         <v>45864</v>
       </c>
-      <c r="E55">
+      <c r="E55" s="4">
         <v>17</v>
       </c>
       <c r="F55" t="s">
@@ -2093,7 +2203,7 @@
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A56" s="5" t="s">
+      <c r="A56" t="s">
         <v>117</v>
       </c>
       <c r="B56" t="s">
@@ -2105,7 +2215,7 @@
       <c r="D56" s="2">
         <v>45867</v>
       </c>
-      <c r="E56" t="s">
+      <c r="E56" s="4" t="s">
         <v>70</v>
       </c>
       <c r="F56" t="s">
@@ -2116,7 +2226,7 @@
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A57" s="5" t="s">
+      <c r="A57" t="s">
         <v>118</v>
       </c>
       <c r="B57" t="s">
@@ -2128,7 +2238,7 @@
       <c r="D57" s="2">
         <v>45872</v>
       </c>
-      <c r="E57">
+      <c r="E57" s="4">
         <v>18</v>
       </c>
       <c r="F57" t="s">
@@ -2139,7 +2249,7 @@
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A58" s="5" t="s">
+      <c r="A58" t="s">
         <v>119</v>
       </c>
       <c r="B58" t="s">
@@ -2151,7 +2261,7 @@
       <c r="D58" s="2">
         <v>45883</v>
       </c>
-      <c r="E58" t="s">
+      <c r="E58" s="4" t="s">
         <v>70</v>
       </c>
       <c r="F58" t="s">
@@ -2162,7 +2272,7 @@
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A59" s="5" t="s">
+      <c r="A59" t="s">
         <v>120</v>
       </c>
       <c r="B59" t="s">
@@ -2174,7 +2284,7 @@
       <c r="D59" s="2">
         <v>45886</v>
       </c>
-      <c r="E59">
+      <c r="E59" s="4">
         <v>20</v>
       </c>
       <c r="F59" t="s">
@@ -2185,7 +2295,7 @@
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A60" s="5" t="s">
+      <c r="A60" t="s">
         <v>121</v>
       </c>
       <c r="B60" t="s">
@@ -2197,7 +2307,7 @@
       <c r="D60" s="2">
         <v>45899</v>
       </c>
-      <c r="E60">
+      <c r="E60" s="4">
         <v>22</v>
       </c>
       <c r="F60" t="s">
@@ -2208,7 +2318,7 @@
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A61" s="5" t="s">
+      <c r="A61" t="s">
         <v>122</v>
       </c>
       <c r="B61" t="s">
@@ -2220,7 +2330,7 @@
       <c r="D61" s="2">
         <v>45911</v>
       </c>
-      <c r="E61" t="s">
+      <c r="E61" s="4" t="s">
         <v>71</v>
       </c>
       <c r="F61" t="s">
@@ -2231,7 +2341,7 @@
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A62" s="5" t="s">
+      <c r="A62" t="s">
         <v>123</v>
       </c>
       <c r="B62" t="s">
@@ -2243,7 +2353,7 @@
       <c r="D62" s="2">
         <v>45917</v>
       </c>
-      <c r="E62">
+      <c r="E62" s="4">
         <v>12</v>
       </c>
       <c r="F62" t="s">
@@ -2254,7 +2364,7 @@
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A63" s="5" t="s">
+      <c r="A63" t="s">
         <v>125</v>
       </c>
       <c r="B63" t="s">
@@ -2266,7 +2376,7 @@
       <c r="D63" s="2">
         <v>45920</v>
       </c>
-      <c r="E63">
+      <c r="E63" s="4">
         <v>24</v>
       </c>
       <c r="F63" t="s">
@@ -2277,33 +2387,33 @@
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A64" s="5" t="s">
+      <c r="A64" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="B64" t="s">
-        <v>8</v>
-      </c>
-      <c r="C64" t="s">
+      <c r="B64" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C64" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D64" s="2">
+      <c r="D64" s="7">
         <v>45931</v>
       </c>
-      <c r="E64">
+      <c r="E64" s="8">
         <v>26</v>
       </c>
-      <c r="F64" t="s">
+      <c r="F64" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="G64" s="3">
+      <c r="G64" s="9">
         <v>0.89583333333333337</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A65" s="5" t="s">
+      <c r="A65" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="B65" t="s">
+      <c r="B65" s="11" t="s">
         <v>8</v>
       </c>
       <c r="C65" t="s">
@@ -2312,7 +2422,7 @@
       <c r="D65" s="2">
         <v>45945</v>
       </c>
-      <c r="E65">
+      <c r="E65" s="4">
         <v>28</v>
       </c>
       <c r="F65" t="s">
@@ -2320,6 +2430,420 @@
       </c>
       <c r="G65" s="3">
         <v>0.8125</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A66" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="B66" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C66" t="s">
+        <v>148</v>
+      </c>
+      <c r="D66" s="2">
+        <v>45956</v>
+      </c>
+      <c r="E66" s="4">
+        <v>30</v>
+      </c>
+      <c r="F66" t="s">
+        <v>13</v>
+      </c>
+      <c r="G66" s="3">
+        <v>0.66666666666666663</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A67" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="B67" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C67" t="s">
+        <v>40</v>
+      </c>
+      <c r="D67" s="2">
+        <v>45966</v>
+      </c>
+      <c r="E67" s="4">
+        <v>32</v>
+      </c>
+      <c r="F67" t="s">
+        <v>21</v>
+      </c>
+      <c r="G67" s="3">
+        <v>0.8125</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A68" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="B68" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C68" t="s">
+        <v>150</v>
+      </c>
+      <c r="D68" s="2">
+        <v>45979</v>
+      </c>
+      <c r="E68" s="4">
+        <v>34</v>
+      </c>
+      <c r="F68" t="s">
+        <v>18</v>
+      </c>
+      <c r="G68" s="3">
+        <v>0.85416666666666663</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A69" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="B69" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C69" t="s">
+        <v>149</v>
+      </c>
+      <c r="D69" s="2">
+        <v>45983</v>
+      </c>
+      <c r="E69" s="4">
+        <v>35</v>
+      </c>
+      <c r="F69" t="s">
+        <v>30</v>
+      </c>
+      <c r="G69" s="3">
+        <v>0.8125</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A70" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="B70" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C70" t="s">
+        <v>36</v>
+      </c>
+      <c r="D70" s="2">
+        <v>45998</v>
+      </c>
+      <c r="E70" s="4">
+        <v>38</v>
+      </c>
+      <c r="F70" t="s">
+        <v>13</v>
+      </c>
+      <c r="G70" s="3">
+        <v>0.66666666666666663</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>137</v>
+      </c>
+      <c r="B71" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C71" t="s">
+        <v>86</v>
+      </c>
+      <c r="D71" s="2">
+        <v>46043</v>
+      </c>
+      <c r="E71" s="4">
+        <v>3</v>
+      </c>
+      <c r="F71" t="s">
+        <v>21</v>
+      </c>
+      <c r="G71" s="3">
+        <v>0.79166666666666663</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
+        <v>138</v>
+      </c>
+      <c r="B72" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C72" t="s">
+        <v>48</v>
+      </c>
+      <c r="D72" s="2">
+        <v>46046</v>
+      </c>
+      <c r="E72" s="4">
+        <v>4</v>
+      </c>
+      <c r="F72" t="s">
+        <v>30</v>
+      </c>
+      <c r="G72" s="3">
+        <v>0.875</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>139</v>
+      </c>
+      <c r="B73" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C73" t="s">
+        <v>32</v>
+      </c>
+      <c r="D73" s="2">
+        <v>46051</v>
+      </c>
+      <c r="E73" s="4">
+        <v>1</v>
+      </c>
+      <c r="F73" t="s">
+        <v>10</v>
+      </c>
+      <c r="G73" s="3">
+        <v>0.89583333333333337</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>140</v>
+      </c>
+      <c r="B74" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C74" t="s">
+        <v>17</v>
+      </c>
+      <c r="D74" s="2">
+        <v>46054</v>
+      </c>
+      <c r="E74" s="4">
+        <v>5</v>
+      </c>
+      <c r="F74" t="s">
+        <v>13</v>
+      </c>
+      <c r="G74" s="3">
+        <v>0.85416666666666663</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>141</v>
+      </c>
+      <c r="B75" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C75" t="s">
+        <v>34</v>
+      </c>
+      <c r="D75" s="2">
+        <v>46068</v>
+      </c>
+      <c r="E75" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="F75" t="s">
+        <v>13</v>
+      </c>
+      <c r="G75" s="3">
+        <v>0.72916666666666663</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
+        <v>142</v>
+      </c>
+      <c r="B76" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C76" t="s">
+        <v>152</v>
+      </c>
+      <c r="D76" s="2">
+        <v>46078</v>
+      </c>
+      <c r="E76" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="F76" t="s">
+        <v>21</v>
+      </c>
+      <c r="G76" s="3">
+        <v>0.89583333333333337</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
+        <v>143</v>
+      </c>
+      <c r="B77" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C77" t="s">
+        <v>51</v>
+      </c>
+      <c r="D77" s="2">
+        <v>46081</v>
+      </c>
+      <c r="E77" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="F77" t="s">
+        <v>30</v>
+      </c>
+      <c r="G77" s="3">
+        <v>0.8125</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>144</v>
+      </c>
+      <c r="B78" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C78" t="s">
+        <v>48</v>
+      </c>
+      <c r="D78" s="2">
+        <v>46088</v>
+      </c>
+      <c r="E78" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="F78" t="s">
+        <v>30</v>
+      </c>
+      <c r="G78" s="3">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>145</v>
+      </c>
+      <c r="B79" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C79" t="s">
+        <v>151</v>
+      </c>
+      <c r="D79" s="2">
+        <v>46091</v>
+      </c>
+      <c r="E79" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="F79" t="s">
+        <v>18</v>
+      </c>
+      <c r="G79" s="3">
+        <v>0.89583333333333337</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>146</v>
+      </c>
+      <c r="B80" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C80" t="s">
+        <v>34</v>
+      </c>
+      <c r="D80" s="2">
+        <v>46095</v>
+      </c>
+      <c r="E80" s="4">
+        <v>6</v>
+      </c>
+      <c r="F80" t="s">
+        <v>30</v>
+      </c>
+      <c r="G80" s="3">
+        <v>0.85416666666666663</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
+        <v>147</v>
+      </c>
+      <c r="B81" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C81" t="s">
+        <v>124</v>
+      </c>
+      <c r="D81" s="2">
+        <v>46113</v>
+      </c>
+      <c r="E81" s="4">
+        <v>9</v>
+      </c>
+      <c r="F81" t="s">
+        <v>21</v>
+      </c>
+      <c r="G81" s="3">
+        <v>0.8125</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
+        <v>156</v>
+      </c>
+      <c r="B82" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="C82" t="s">
+        <v>155</v>
+      </c>
+      <c r="D82" s="2">
+        <v>46121</v>
+      </c>
+      <c r="E82" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="F82" t="s">
+        <v>10</v>
+      </c>
+      <c r="G82" s="3">
+        <v>0.79166666666666663</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>157</v>
+      </c>
+      <c r="B83" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C83" t="s">
+        <v>154</v>
+      </c>
+      <c r="D83" s="2">
+        <v>46124</v>
+      </c>
+      <c r="E83" s="4">
+        <v>11</v>
+      </c>
+      <c r="F83" t="s">
+        <v>13</v>
+      </c>
+      <c r="G83" s="3">
+        <v>0.66666666666666663</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Apply light design system + sidebar layout + data update
Design (light theme):
- tokens.js: #F8FAFC base, white cards, slate palette, gold #C5A059
- index.html: Space Grotesk + Inter fonts, light bg, slate scrollbar
- App.jsx: sidebar 272px (white), glassmorphism header, dynamic page titles
- Card/KPICard/Tooltip: white cards borderRadius 24px, slate-200 border, ambient shadow

Data update (xlsx → data.js):
- dPartidas, dTimes, fDespesas, fFacial, fIngressos atualizados
- 82 partidas | público total 1.610.092 | ticket médio R$ 31,41 | sócios 62,6%

Page fixes (color-only, features preserved):
- ChampionshipReport: rows #F8FAFC/#ffffff, text C.t1/t2/t3, Nao Socio #64748b
- PL: rows light, total row #0F172A, cats #F1F5F9, C.red/green/t3 for values
- Comparativo: 2024 series #94a3b8 (slate-400)

https://claude.ai/code/session_01Bb3ciycnMnk9Z7WYwsqMvC
</commit_message>
<xml_diff>
--- a/dPartidas.xlsx
+++ b/dPartidas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="EstaPastaDeTrabalho" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://safbotafogo-my.sharepoint.com/personal/pedro_arruda_safbfr_com_br/Documents/BI/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://safbotafogo-my.sharepoint.com/personal/pedro_arruda_safbfr_com_br/Documents/Área de Trabalho/dash-ticket/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="296" documentId="8_{E25D5179-CBFE-42C3-9E8D-799BA19C3FB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A72B6E0D-2D08-47BD-AD4B-0FC36731CE92}"/>
+  <xr:revisionPtr revIDLastSave="477" documentId="8_{E25D5179-CBFE-42C3-9E8D-799BA19C3FB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15D5C576-7611-44B6-AFD0-EE56B32D2144}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E1B40A1D-D5F1-4DC5-B00D-B969B491F639}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E1B40A1D-D5F1-4DC5-B00D-B969B491F639}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha3" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="158">
   <si>
     <t>ID_PARTIDA</t>
   </si>
@@ -423,6 +423,96 @@
   </si>
   <si>
     <t>2025.10.15-CAMBR2-28</t>
+  </si>
+  <si>
+    <t>3° Fase</t>
+  </si>
+  <si>
+    <t>Quartas</t>
+  </si>
+  <si>
+    <t>SEMIS - TR</t>
+  </si>
+  <si>
+    <t>FINAL - TR</t>
+  </si>
+  <si>
+    <t>2025.10.26-CAMBR2-30</t>
+  </si>
+  <si>
+    <t>2025.11.05-CAMBR2-32</t>
+  </si>
+  <si>
+    <t>2025.11.18-CAMBR2-34</t>
+  </si>
+  <si>
+    <t>2025.11.22-CAMBR2-35</t>
+  </si>
+  <si>
+    <t>2025.12.07-CAMBR2-38</t>
+  </si>
+  <si>
+    <t>2026.01.21-CAMCA4-3</t>
+  </si>
+  <si>
+    <t>2026.01.24-CAMCA4-4</t>
+  </si>
+  <si>
+    <t>2026.01.29-CAMBR2-1</t>
+  </si>
+  <si>
+    <t>2026.02.01-CAMCA4-5</t>
+  </si>
+  <si>
+    <t>2026.02.15-CAMCA4-Quartas</t>
+  </si>
+  <si>
+    <t>2026.02.25-CAMLI5-2° FASE</t>
+  </si>
+  <si>
+    <t>2026.02.28-CAMCA4-SEMIS - TR</t>
+  </si>
+  <si>
+    <t>2026.03.07-CAMCA4-FINAL - TR</t>
+  </si>
+  <si>
+    <t>2026.03.10-CAMLI5-3° Fase</t>
+  </si>
+  <si>
+    <t>2026.03.14-CAMBR2-6</t>
+  </si>
+  <si>
+    <t>2026.04.01-CAMBR2-9</t>
+  </si>
+  <si>
+    <t>7SABRSP</t>
+  </si>
+  <si>
+    <t>10GRBRRS</t>
+  </si>
+  <si>
+    <t>13SPBRPE</t>
+  </si>
+  <si>
+    <t>93BAECGU</t>
+  </si>
+  <si>
+    <t>123NABOPO</t>
+  </si>
+  <si>
+    <t>CAMSU6</t>
+  </si>
+  <si>
+    <t>12COBRPR</t>
+  </si>
+  <si>
+    <t>115CAVECA</t>
+  </si>
+  <si>
+    <t>2026.04.09-CAMSU6-FG</t>
+  </si>
+  <si>
+    <t>2026.04.12-CAMBR2-11</t>
   </si>
 </sst>
 </file>
@@ -452,12 +542,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -472,7 +574,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -480,6 +582,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -816,13 +928,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2921BBCD-6E27-463C-B492-0BF065778598}">
   <sheetPr codeName="Planilha1"/>
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G83"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.81640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.90625" style="4" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.81640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.81640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -840,7 +953,7 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -978,7 +1091,7 @@
       <c r="D7" s="2">
         <v>45350</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="4" t="s">
         <v>67</v>
       </c>
       <c r="F7" t="s">
@@ -1001,7 +1114,7 @@
       <c r="D8" s="2">
         <v>45357</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="4" t="s">
         <v>68</v>
       </c>
       <c r="F8" t="s">
@@ -1070,7 +1183,7 @@
       <c r="D11" s="2">
         <v>45385</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="4" t="s">
         <v>69</v>
       </c>
       <c r="F11" t="s">
@@ -1139,7 +1252,7 @@
       <c r="D14" s="2">
         <v>45406</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="4" t="s">
         <v>69</v>
       </c>
       <c r="F14" t="s">
@@ -1162,7 +1275,7 @@
       <c r="D15" s="2">
         <v>45414</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="4" t="s">
         <v>68</v>
       </c>
       <c r="F15" t="s">
@@ -1208,7 +1321,7 @@
       <c r="D17" s="2">
         <v>45420</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="4" t="s">
         <v>69</v>
       </c>
       <c r="F17" t="s">
@@ -1392,7 +1505,7 @@
       <c r="D25" s="2">
         <v>45503</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" s="4" t="s">
         <v>70</v>
       </c>
       <c r="F25" t="s">
@@ -1406,16 +1519,13 @@
       <c r="A26" t="s">
         <v>79</v>
       </c>
-      <c r="B26" t="s">
-        <v>73</v>
-      </c>
       <c r="C26" t="s">
         <v>27</v>
       </c>
       <c r="D26" s="2">
         <v>45518</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E26" s="4" t="s">
         <v>70</v>
       </c>
       <c r="F26" t="s">
@@ -1507,7 +1617,7 @@
       <c r="D30" s="2">
         <v>45553</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E30" s="4" t="s">
         <v>71</v>
       </c>
       <c r="F30" t="s">
@@ -1530,7 +1640,7 @@
       <c r="D31" s="2">
         <v>45560</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E31" s="4" t="s">
         <v>71</v>
       </c>
       <c r="F31" t="s">
@@ -1553,7 +1663,7 @@
       <c r="D32" s="2">
         <v>45583</v>
       </c>
-      <c r="E32">
+      <c r="E32" s="4">
         <v>30</v>
       </c>
       <c r="F32" t="s">
@@ -1576,7 +1686,7 @@
       <c r="D33" s="2">
         <v>45588</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E33" s="4" t="s">
         <v>72</v>
       </c>
       <c r="F33" t="s">
@@ -1599,7 +1709,7 @@
       <c r="D34" s="2">
         <v>45595</v>
       </c>
-      <c r="E34" t="s">
+      <c r="E34" s="4" t="s">
         <v>72</v>
       </c>
       <c r="F34" t="s">
@@ -1714,7 +1824,7 @@
       <c r="D39" s="2">
         <v>45668</v>
       </c>
-      <c r="E39">
+      <c r="E39" s="4">
         <v>1</v>
       </c>
       <c r="F39" t="s">
@@ -1737,7 +1847,7 @@
       <c r="D40" s="2">
         <v>45671</v>
       </c>
-      <c r="E40">
+      <c r="E40" s="4">
         <v>2</v>
       </c>
       <c r="F40" t="s">
@@ -1760,7 +1870,7 @@
       <c r="D41" s="2">
         <v>45679</v>
       </c>
-      <c r="E41">
+      <c r="E41" s="4">
         <v>4</v>
       </c>
       <c r="F41" t="s">
@@ -1783,7 +1893,7 @@
       <c r="D42" s="2">
         <v>45683</v>
       </c>
-      <c r="E42">
+      <c r="E42" s="4">
         <v>5</v>
       </c>
       <c r="F42" t="s">
@@ -1806,7 +1916,7 @@
       <c r="D43" s="2">
         <v>45686</v>
       </c>
-      <c r="E43">
+      <c r="E43" s="4">
         <v>6</v>
       </c>
       <c r="F43" t="s">
@@ -1817,7 +1927,7 @@
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A44" s="5" t="s">
+      <c r="A44" t="s">
         <v>107</v>
       </c>
       <c r="B44" t="s">
@@ -1829,7 +1939,7 @@
       <c r="D44" s="2">
         <v>45715</v>
       </c>
-      <c r="E44" t="s">
+      <c r="E44" s="4" t="s">
         <v>104</v>
       </c>
       <c r="F44" t="s">
@@ -1840,7 +1950,7 @@
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A45" s="5" t="s">
+      <c r="A45" t="s">
         <v>96</v>
       </c>
       <c r="B45" t="s">
@@ -1852,7 +1962,7 @@
       <c r="D45" s="2">
         <v>45752</v>
       </c>
-      <c r="E45">
+      <c r="E45" s="4">
         <v>2</v>
       </c>
       <c r="F45" t="s">
@@ -1863,7 +1973,7 @@
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A46" s="5" t="s">
+      <c r="A46" t="s">
         <v>97</v>
       </c>
       <c r="B46" t="s">
@@ -1875,7 +1985,7 @@
       <c r="D46" s="2">
         <v>45755</v>
       </c>
-      <c r="E46">
+      <c r="E46" s="4">
         <v>2</v>
       </c>
       <c r="F46" t="s">
@@ -1886,7 +1996,7 @@
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A47" s="5" t="s">
+      <c r="A47" t="s">
         <v>98</v>
       </c>
       <c r="B47" t="s">
@@ -1898,7 +2008,7 @@
       <c r="D47" s="2">
         <v>45763</v>
       </c>
-      <c r="E47">
+      <c r="E47" s="4">
         <v>4</v>
       </c>
       <c r="F47" t="s">
@@ -1909,7 +2019,7 @@
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A48" s="5" t="s">
+      <c r="A48" t="s">
         <v>99</v>
       </c>
       <c r="B48" t="s">
@@ -1921,7 +2031,7 @@
       <c r="D48" s="2">
         <v>45773</v>
       </c>
-      <c r="E48">
+      <c r="E48" s="4">
         <v>6</v>
       </c>
       <c r="F48" t="s">
@@ -1932,7 +2042,7 @@
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A49" s="5" t="s">
+      <c r="A49" t="s">
         <v>100</v>
       </c>
       <c r="B49" t="s">
@@ -1944,7 +2054,7 @@
       <c r="D49" s="2">
         <v>45777</v>
       </c>
-      <c r="E49" t="s">
+      <c r="E49" s="4" t="s">
         <v>68</v>
       </c>
       <c r="F49" t="s">
@@ -1955,7 +2065,7 @@
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A50" s="5" t="s">
+      <c r="A50" t="s">
         <v>106</v>
       </c>
       <c r="B50" t="s">
@@ -1967,7 +2077,7 @@
       <c r="D50" s="2">
         <v>45788</v>
       </c>
-      <c r="E50">
+      <c r="E50" s="4">
         <v>8</v>
       </c>
       <c r="F50" t="s">
@@ -1978,7 +2088,7 @@
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A51" s="5" t="s">
+      <c r="A51" t="s">
         <v>109</v>
       </c>
       <c r="B51" t="s">
@@ -1990,7 +2100,7 @@
       <c r="D51" s="2">
         <v>45791</v>
       </c>
-      <c r="E51">
+      <c r="E51" s="4">
         <v>5</v>
       </c>
       <c r="F51" t="s">
@@ -2001,7 +2111,7 @@
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A52" s="5" t="s">
+      <c r="A52" t="s">
         <v>111</v>
       </c>
       <c r="B52" t="s">
@@ -2013,7 +2123,7 @@
       <c r="D52" s="2">
         <v>45804</v>
       </c>
-      <c r="E52">
+      <c r="E52" s="4">
         <v>6</v>
       </c>
       <c r="F52" t="s">
@@ -2024,7 +2134,7 @@
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A53" s="5" t="s">
+      <c r="A53" t="s">
         <v>114</v>
       </c>
       <c r="B53" t="s">
@@ -2036,7 +2146,7 @@
       <c r="D53" s="2">
         <v>45812</v>
       </c>
-      <c r="E53">
+      <c r="E53" s="4">
         <v>10</v>
       </c>
       <c r="F53" t="s">
@@ -2047,7 +2157,7 @@
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A54" s="5" t="s">
+      <c r="A54" t="s">
         <v>115</v>
       </c>
       <c r="B54" t="s">
@@ -2059,7 +2169,7 @@
       <c r="D54" s="2">
         <v>45854</v>
       </c>
-      <c r="E54">
+      <c r="E54" s="4">
         <v>14</v>
       </c>
       <c r="F54" t="s">
@@ -2070,7 +2180,7 @@
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A55" s="5" t="s">
+      <c r="A55" t="s">
         <v>116</v>
       </c>
       <c r="B55" t="s">
@@ -2082,7 +2192,7 @@
       <c r="D55" s="2">
         <v>45864</v>
       </c>
-      <c r="E55">
+      <c r="E55" s="4">
         <v>17</v>
       </c>
       <c r="F55" t="s">
@@ -2093,7 +2203,7 @@
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A56" s="5" t="s">
+      <c r="A56" t="s">
         <v>117</v>
       </c>
       <c r="B56" t="s">
@@ -2105,7 +2215,7 @@
       <c r="D56" s="2">
         <v>45867</v>
       </c>
-      <c r="E56" t="s">
+      <c r="E56" s="4" t="s">
         <v>70</v>
       </c>
       <c r="F56" t="s">
@@ -2116,7 +2226,7 @@
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A57" s="5" t="s">
+      <c r="A57" t="s">
         <v>118</v>
       </c>
       <c r="B57" t="s">
@@ -2128,7 +2238,7 @@
       <c r="D57" s="2">
         <v>45872</v>
       </c>
-      <c r="E57">
+      <c r="E57" s="4">
         <v>18</v>
       </c>
       <c r="F57" t="s">
@@ -2139,7 +2249,7 @@
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A58" s="5" t="s">
+      <c r="A58" t="s">
         <v>119</v>
       </c>
       <c r="B58" t="s">
@@ -2151,7 +2261,7 @@
       <c r="D58" s="2">
         <v>45883</v>
       </c>
-      <c r="E58" t="s">
+      <c r="E58" s="4" t="s">
         <v>70</v>
       </c>
       <c r="F58" t="s">
@@ -2162,7 +2272,7 @@
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A59" s="5" t="s">
+      <c r="A59" t="s">
         <v>120</v>
       </c>
       <c r="B59" t="s">
@@ -2174,7 +2284,7 @@
       <c r="D59" s="2">
         <v>45886</v>
       </c>
-      <c r="E59">
+      <c r="E59" s="4">
         <v>20</v>
       </c>
       <c r="F59" t="s">
@@ -2185,7 +2295,7 @@
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A60" s="5" t="s">
+      <c r="A60" t="s">
         <v>121</v>
       </c>
       <c r="B60" t="s">
@@ -2197,7 +2307,7 @@
       <c r="D60" s="2">
         <v>45899</v>
       </c>
-      <c r="E60">
+      <c r="E60" s="4">
         <v>22</v>
       </c>
       <c r="F60" t="s">
@@ -2208,7 +2318,7 @@
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A61" s="5" t="s">
+      <c r="A61" t="s">
         <v>122</v>
       </c>
       <c r="B61" t="s">
@@ -2220,7 +2330,7 @@
       <c r="D61" s="2">
         <v>45911</v>
       </c>
-      <c r="E61" t="s">
+      <c r="E61" s="4" t="s">
         <v>71</v>
       </c>
       <c r="F61" t="s">
@@ -2231,7 +2341,7 @@
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A62" s="5" t="s">
+      <c r="A62" t="s">
         <v>123</v>
       </c>
       <c r="B62" t="s">
@@ -2243,7 +2353,7 @@
       <c r="D62" s="2">
         <v>45917</v>
       </c>
-      <c r="E62">
+      <c r="E62" s="4">
         <v>12</v>
       </c>
       <c r="F62" t="s">
@@ -2254,7 +2364,7 @@
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A63" s="5" t="s">
+      <c r="A63" t="s">
         <v>125</v>
       </c>
       <c r="B63" t="s">
@@ -2266,7 +2376,7 @@
       <c r="D63" s="2">
         <v>45920</v>
       </c>
-      <c r="E63">
+      <c r="E63" s="4">
         <v>24</v>
       </c>
       <c r="F63" t="s">
@@ -2277,33 +2387,33 @@
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A64" s="5" t="s">
+      <c r="A64" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="B64" t="s">
-        <v>8</v>
-      </c>
-      <c r="C64" t="s">
+      <c r="B64" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C64" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D64" s="2">
+      <c r="D64" s="7">
         <v>45931</v>
       </c>
-      <c r="E64">
+      <c r="E64" s="8">
         <v>26</v>
       </c>
-      <c r="F64" t="s">
+      <c r="F64" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="G64" s="3">
+      <c r="G64" s="9">
         <v>0.89583333333333337</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A65" s="5" t="s">
+      <c r="A65" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="B65" t="s">
+      <c r="B65" s="11" t="s">
         <v>8</v>
       </c>
       <c r="C65" t="s">
@@ -2312,7 +2422,7 @@
       <c r="D65" s="2">
         <v>45945</v>
       </c>
-      <c r="E65">
+      <c r="E65" s="4">
         <v>28</v>
       </c>
       <c r="F65" t="s">
@@ -2320,6 +2430,420 @@
       </c>
       <c r="G65" s="3">
         <v>0.8125</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A66" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="B66" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C66" t="s">
+        <v>148</v>
+      </c>
+      <c r="D66" s="2">
+        <v>45956</v>
+      </c>
+      <c r="E66" s="4">
+        <v>30</v>
+      </c>
+      <c r="F66" t="s">
+        <v>13</v>
+      </c>
+      <c r="G66" s="3">
+        <v>0.66666666666666663</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A67" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="B67" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C67" t="s">
+        <v>40</v>
+      </c>
+      <c r="D67" s="2">
+        <v>45966</v>
+      </c>
+      <c r="E67" s="4">
+        <v>32</v>
+      </c>
+      <c r="F67" t="s">
+        <v>21</v>
+      </c>
+      <c r="G67" s="3">
+        <v>0.8125</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A68" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="B68" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C68" t="s">
+        <v>150</v>
+      </c>
+      <c r="D68" s="2">
+        <v>45979</v>
+      </c>
+      <c r="E68" s="4">
+        <v>34</v>
+      </c>
+      <c r="F68" t="s">
+        <v>18</v>
+      </c>
+      <c r="G68" s="3">
+        <v>0.85416666666666663</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A69" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="B69" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C69" t="s">
+        <v>149</v>
+      </c>
+      <c r="D69" s="2">
+        <v>45983</v>
+      </c>
+      <c r="E69" s="4">
+        <v>35</v>
+      </c>
+      <c r="F69" t="s">
+        <v>30</v>
+      </c>
+      <c r="G69" s="3">
+        <v>0.8125</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A70" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="B70" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C70" t="s">
+        <v>36</v>
+      </c>
+      <c r="D70" s="2">
+        <v>45998</v>
+      </c>
+      <c r="E70" s="4">
+        <v>38</v>
+      </c>
+      <c r="F70" t="s">
+        <v>13</v>
+      </c>
+      <c r="G70" s="3">
+        <v>0.66666666666666663</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>137</v>
+      </c>
+      <c r="B71" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C71" t="s">
+        <v>86</v>
+      </c>
+      <c r="D71" s="2">
+        <v>46043</v>
+      </c>
+      <c r="E71" s="4">
+        <v>3</v>
+      </c>
+      <c r="F71" t="s">
+        <v>21</v>
+      </c>
+      <c r="G71" s="3">
+        <v>0.79166666666666663</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
+        <v>138</v>
+      </c>
+      <c r="B72" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C72" t="s">
+        <v>48</v>
+      </c>
+      <c r="D72" s="2">
+        <v>46046</v>
+      </c>
+      <c r="E72" s="4">
+        <v>4</v>
+      </c>
+      <c r="F72" t="s">
+        <v>30</v>
+      </c>
+      <c r="G72" s="3">
+        <v>0.875</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>139</v>
+      </c>
+      <c r="B73" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C73" t="s">
+        <v>32</v>
+      </c>
+      <c r="D73" s="2">
+        <v>46051</v>
+      </c>
+      <c r="E73" s="4">
+        <v>1</v>
+      </c>
+      <c r="F73" t="s">
+        <v>10</v>
+      </c>
+      <c r="G73" s="3">
+        <v>0.89583333333333337</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>140</v>
+      </c>
+      <c r="B74" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C74" t="s">
+        <v>17</v>
+      </c>
+      <c r="D74" s="2">
+        <v>46054</v>
+      </c>
+      <c r="E74" s="4">
+        <v>5</v>
+      </c>
+      <c r="F74" t="s">
+        <v>13</v>
+      </c>
+      <c r="G74" s="3">
+        <v>0.85416666666666663</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>141</v>
+      </c>
+      <c r="B75" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C75" t="s">
+        <v>34</v>
+      </c>
+      <c r="D75" s="2">
+        <v>46068</v>
+      </c>
+      <c r="E75" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="F75" t="s">
+        <v>13</v>
+      </c>
+      <c r="G75" s="3">
+        <v>0.72916666666666663</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
+        <v>142</v>
+      </c>
+      <c r="B76" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C76" t="s">
+        <v>152</v>
+      </c>
+      <c r="D76" s="2">
+        <v>46078</v>
+      </c>
+      <c r="E76" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="F76" t="s">
+        <v>21</v>
+      </c>
+      <c r="G76" s="3">
+        <v>0.89583333333333337</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
+        <v>143</v>
+      </c>
+      <c r="B77" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C77" t="s">
+        <v>51</v>
+      </c>
+      <c r="D77" s="2">
+        <v>46081</v>
+      </c>
+      <c r="E77" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="F77" t="s">
+        <v>30</v>
+      </c>
+      <c r="G77" s="3">
+        <v>0.8125</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>144</v>
+      </c>
+      <c r="B78" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C78" t="s">
+        <v>48</v>
+      </c>
+      <c r="D78" s="2">
+        <v>46088</v>
+      </c>
+      <c r="E78" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="F78" t="s">
+        <v>30</v>
+      </c>
+      <c r="G78" s="3">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>145</v>
+      </c>
+      <c r="B79" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C79" t="s">
+        <v>151</v>
+      </c>
+      <c r="D79" s="2">
+        <v>46091</v>
+      </c>
+      <c r="E79" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="F79" t="s">
+        <v>18</v>
+      </c>
+      <c r="G79" s="3">
+        <v>0.89583333333333337</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>146</v>
+      </c>
+      <c r="B80" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C80" t="s">
+        <v>34</v>
+      </c>
+      <c r="D80" s="2">
+        <v>46095</v>
+      </c>
+      <c r="E80" s="4">
+        <v>6</v>
+      </c>
+      <c r="F80" t="s">
+        <v>30</v>
+      </c>
+      <c r="G80" s="3">
+        <v>0.85416666666666663</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
+        <v>147</v>
+      </c>
+      <c r="B81" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C81" t="s">
+        <v>124</v>
+      </c>
+      <c r="D81" s="2">
+        <v>46113</v>
+      </c>
+      <c r="E81" s="4">
+        <v>9</v>
+      </c>
+      <c r="F81" t="s">
+        <v>21</v>
+      </c>
+      <c r="G81" s="3">
+        <v>0.8125</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
+        <v>156</v>
+      </c>
+      <c r="B82" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="C82" t="s">
+        <v>155</v>
+      </c>
+      <c r="D82" s="2">
+        <v>46121</v>
+      </c>
+      <c r="E82" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="F82" t="s">
+        <v>10</v>
+      </c>
+      <c r="G82" s="3">
+        <v>0.79166666666666663</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>157</v>
+      </c>
+      <c r="B83" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C83" t="s">
+        <v>154</v>
+      </c>
+      <c r="D83" s="2">
+        <v>46124</v>
+      </c>
+      <c r="E83" s="4">
+        <v>11</v>
+      </c>
+      <c r="F83" t="s">
+        <v>13</v>
+      </c>
+      <c r="G83" s="3">
+        <v>0.66666666666666663</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: atualiza xlsx e regenera data.js com 82 partidas (+2)
Incorpora arquivos mais completos de dados:
- dPartidas/fIngressos: 82 partidas (era 80)
- fEstacionamento: 67 partidas (era 54)
- fFirezone/fArenaKids: 68 partidas (era 55)
- fA&B: 64 partidas (era 54)
fDespesas, fFacial, fBordero, fAcomodacao mantidos (cobertura maior na branch atual).

https://claude.ai/code/session_01KkiyBKLV3FeeQwKRqX37Yb
</commit_message>
<xml_diff>
--- a/dPartidas.xlsx
+++ b/dPartidas.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="EstaPastaDeTrabalho" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://safbotafogo-my.sharepoint.com/personal/pedro_arruda_safbfr_com_br/Documents/Área de Trabalho/dash-ticket/dash-ticket/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://safbotafogo-my.sharepoint.com/personal/pedro_arruda_safbfr_com_br/Documents/Área de Trabalho/dash-ticket/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="498" documentId="8_{E25D5179-CBFE-42C3-9E8D-799BA19C3FB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8179ABC-46C4-4CEB-8A71-F247D13674EE}"/>
+  <xr:revisionPtr revIDLastSave="477" documentId="8_{E25D5179-CBFE-42C3-9E8D-799BA19C3FB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15D5C576-7611-44B6-AFD0-EE56B32D2144}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E1B40A1D-D5F1-4DC5-B00D-B969B491F639}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Planilha3" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha3!$A$1:$G$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha3!$A$1:$G$64</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="158">
   <si>
     <t>ID_PARTIDA</t>
   </si>
@@ -285,6 +285,12 @@
   </si>
   <si>
     <t>2024.10.23-CAMLI5-SEMIS</t>
+  </si>
+  <si>
+    <t>2024.09.25-CAMLI5-QUARTAS</t>
+  </si>
+  <si>
+    <t>2024.10.30-CAMLI5-SEMIS</t>
   </si>
   <si>
     <t>Sexta-feira</t>
@@ -568,7 +574,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -586,6 +592,7 @@
     </xf>
     <xf numFmtId="20" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -921,7 +928,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2921BBCD-6E27-463C-B492-0BF065778598}">
   <sheetPr codeName="Planilha1"/>
-  <dimension ref="A1:G81"/>
+  <dimension ref="A1:G83"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.81640625" bestFit="1" customWidth="1"/>
@@ -1257,10 +1264,10 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B15" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C15" t="s">
         <v>44</v>
@@ -1487,10 +1494,10 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B25" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C25" t="s">
         <v>15</v>
@@ -1512,9 +1519,6 @@
       <c r="A26" t="s">
         <v>79</v>
       </c>
-      <c r="B26" t="s">
-        <v>73</v>
-      </c>
       <c r="C26" t="s">
         <v>27</v>
       </c>
@@ -1625,68 +1629,68 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>106</v>
+        <v>82</v>
       </c>
       <c r="B31" t="s">
-        <v>8</v>
+        <v>73</v>
       </c>
       <c r="C31" t="s">
-        <v>83</v>
+        <v>46</v>
       </c>
       <c r="D31" s="2">
-        <v>45583</v>
-      </c>
-      <c r="E31" s="4">
-        <v>30</v>
+        <v>45560</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>71</v>
       </c>
       <c r="F31" t="s">
-        <v>82</v>
+        <v>21</v>
       </c>
       <c r="G31" s="3">
-        <v>0.83333333333333337</v>
+        <v>0.89583333333333337</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>81</v>
+        <v>108</v>
       </c>
       <c r="B32" t="s">
-        <v>73</v>
+        <v>8</v>
       </c>
       <c r="C32" t="s">
-        <v>66</v>
+        <v>85</v>
       </c>
       <c r="D32" s="2">
-        <v>45588</v>
-      </c>
-      <c r="E32" s="4" t="s">
-        <v>72</v>
+        <v>45583</v>
+      </c>
+      <c r="E32" s="4">
+        <v>30</v>
       </c>
       <c r="F32" t="s">
-        <v>21</v>
+        <v>84</v>
       </c>
       <c r="G32" s="3">
-        <v>0.89583333333333337</v>
+        <v>0.83333333333333337</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>39</v>
+        <v>81</v>
       </c>
       <c r="B33" t="s">
-        <v>8</v>
+        <v>73</v>
       </c>
       <c r="C33" t="s">
-        <v>40</v>
+        <v>66</v>
       </c>
       <c r="D33" s="2">
-        <v>45601</v>
-      </c>
-      <c r="E33" s="4">
-        <v>32</v>
+        <v>45588</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>72</v>
       </c>
       <c r="F33" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G33" s="3">
         <v>0.89583333333333337</v>
@@ -1694,117 +1698,117 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>41</v>
+        <v>83</v>
       </c>
       <c r="B34" t="s">
-        <v>8</v>
+        <v>73</v>
       </c>
       <c r="C34" t="s">
-        <v>42</v>
+        <v>66</v>
       </c>
       <c r="D34" s="2">
-        <v>45605</v>
-      </c>
-      <c r="E34" s="4">
-        <v>33</v>
+        <v>45595</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>72</v>
       </c>
       <c r="F34" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="G34" s="3">
-        <v>0.6875</v>
+        <v>0.89583333333333337</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B35" t="s">
         <v>8</v>
       </c>
       <c r="C35" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="D35" s="2">
-        <v>45619</v>
+        <v>45601</v>
       </c>
       <c r="E35" s="4">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F35" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="G35" s="3">
-        <v>0.8125</v>
+        <v>0.89583333333333337</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B36" t="s">
         <v>8</v>
       </c>
       <c r="C36" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D36" s="2">
-        <v>45634</v>
+        <v>45605</v>
       </c>
       <c r="E36" s="4">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F36" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="G36" s="3">
-        <v>0.66666666666666663</v>
+        <v>0.6875</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>86</v>
+        <v>43</v>
       </c>
       <c r="B37" t="s">
-        <v>52</v>
+        <v>8</v>
       </c>
       <c r="C37" t="s">
-        <v>85</v>
+        <v>44</v>
       </c>
       <c r="D37" s="2">
-        <v>45668</v>
+        <v>45619</v>
       </c>
       <c r="E37" s="4">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="F37" t="s">
         <v>30</v>
       </c>
       <c r="G37" s="3">
-        <v>0.66666666666666663</v>
+        <v>0.8125</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>87</v>
+        <v>45</v>
       </c>
       <c r="B38" t="s">
-        <v>52</v>
+        <v>8</v>
       </c>
       <c r="C38" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D38" s="2">
-        <v>45671</v>
+        <v>45634</v>
       </c>
       <c r="E38" s="4">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="F38" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="G38" s="3">
-        <v>0.8125</v>
+        <v>0.66666666666666663</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
@@ -1815,19 +1819,19 @@
         <v>52</v>
       </c>
       <c r="C39" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D39" s="2">
-        <v>45679</v>
+        <v>45668</v>
       </c>
       <c r="E39" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F39" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="G39" s="3">
-        <v>0.89583333333333337</v>
+        <v>0.66666666666666663</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.35">
@@ -1838,19 +1842,19 @@
         <v>52</v>
       </c>
       <c r="C40" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D40" s="2">
-        <v>45683</v>
+        <v>45671</v>
       </c>
       <c r="E40" s="4">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F40" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="G40" s="3">
-        <v>0.75</v>
+        <v>0.8125</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
@@ -1861,13 +1865,13 @@
         <v>52</v>
       </c>
       <c r="C41" t="s">
-        <v>17</v>
+        <v>86</v>
       </c>
       <c r="D41" s="2">
-        <v>45686</v>
+        <v>45679</v>
       </c>
       <c r="E41" s="4">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F41" t="s">
         <v>21</v>
@@ -1878,71 +1882,71 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>105</v>
+        <v>91</v>
       </c>
       <c r="B42" t="s">
-        <v>103</v>
+        <v>52</v>
       </c>
       <c r="C42" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
       <c r="D42" s="2">
-        <v>45715</v>
-      </c>
-      <c r="E42" s="4" t="s">
-        <v>102</v>
+        <v>45683</v>
+      </c>
+      <c r="E42" s="4">
+        <v>5</v>
       </c>
       <c r="F42" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G42" s="3">
-        <v>0.89583333333333337</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B43" t="s">
-        <v>8</v>
+        <v>52</v>
       </c>
       <c r="C43" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D43" s="2">
-        <v>45752</v>
+        <v>45686</v>
       </c>
       <c r="E43" s="4">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F43" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="G43" s="3">
-        <v>0.875</v>
+        <v>0.89583333333333337</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="B44" t="s">
-        <v>73</v>
+        <v>105</v>
       </c>
       <c r="C44" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="D44" s="2">
-        <v>45755</v>
+        <v>45715</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>69</v>
+        <v>104</v>
       </c>
       <c r="F44" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G44" s="3">
-        <v>0.79166666666666663</v>
+        <v>0.89583333333333337</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.35">
@@ -1953,19 +1957,19 @@
         <v>8</v>
       </c>
       <c r="C45" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="D45" s="2">
-        <v>45763</v>
+        <v>45752</v>
       </c>
       <c r="E45" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F45" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="G45" s="3">
-        <v>0.77083333333333337</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
@@ -1973,22 +1977,22 @@
         <v>97</v>
       </c>
       <c r="B46" t="s">
-        <v>8</v>
+        <v>73</v>
       </c>
       <c r="C46" t="s">
-        <v>17</v>
+        <v>94</v>
       </c>
       <c r="D46" s="2">
-        <v>45773</v>
+        <v>45755</v>
       </c>
       <c r="E46" s="4">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F46" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="G46" s="3">
-        <v>0.875</v>
+        <v>0.79166666666666663</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
@@ -1996,134 +2000,134 @@
         <v>98</v>
       </c>
       <c r="B47" t="s">
-        <v>91</v>
+        <v>8</v>
       </c>
       <c r="C47" t="s">
-        <v>93</v>
+        <v>46</v>
       </c>
       <c r="D47" s="2">
-        <v>45777</v>
-      </c>
-      <c r="E47" s="4" t="s">
-        <v>68</v>
+        <v>45763</v>
+      </c>
+      <c r="E47" s="4">
+        <v>4</v>
       </c>
       <c r="F47" t="s">
         <v>21</v>
       </c>
       <c r="G47" s="3">
-        <v>0.79166666666666663</v>
+        <v>0.77083333333333337</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="B48" t="s">
         <v>8</v>
       </c>
       <c r="C48" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="D48" s="2">
-        <v>45788</v>
+        <v>45773</v>
       </c>
       <c r="E48" s="4">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F48" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="G48" s="3">
-        <v>0.83333333333333337</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="B49" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="C49" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="D49" s="2">
-        <v>45791</v>
+        <v>45777</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F49" t="s">
         <v>21</v>
       </c>
       <c r="G49" s="3">
-        <v>0.89583333333333337</v>
+        <v>0.79166666666666663</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B50" t="s">
-        <v>73</v>
+        <v>8</v>
       </c>
       <c r="C50" t="s">
-        <v>110</v>
+        <v>29</v>
       </c>
       <c r="D50" s="2">
-        <v>45804</v>
-      </c>
-      <c r="E50" s="4" t="s">
-        <v>69</v>
+        <v>45788</v>
+      </c>
+      <c r="E50" s="4">
+        <v>8</v>
       </c>
       <c r="F50" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="G50" s="3">
-        <v>0.89583333333333337</v>
+        <v>0.83333333333333337</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B51" t="s">
-        <v>8</v>
+        <v>73</v>
       </c>
       <c r="C51" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D51" s="2">
-        <v>45812</v>
+        <v>45791</v>
       </c>
       <c r="E51" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F51" t="s">
         <v>21</v>
       </c>
       <c r="G51" s="3">
-        <v>0.83333333333333337</v>
+        <v>0.89583333333333337</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B52" t="s">
-        <v>8</v>
+        <v>73</v>
       </c>
       <c r="C52" t="s">
-        <v>44</v>
+        <v>112</v>
       </c>
       <c r="D52" s="2">
-        <v>45854</v>
+        <v>45804</v>
       </c>
       <c r="E52" s="4">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F52" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G52" s="3">
         <v>0.89583333333333337</v>
@@ -2137,19 +2141,19 @@
         <v>8</v>
       </c>
       <c r="C53" t="s">
-        <v>38</v>
+        <v>113</v>
       </c>
       <c r="D53" s="2">
-        <v>45864</v>
+        <v>45812</v>
       </c>
       <c r="E53" s="4">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F53" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="G53" s="3">
-        <v>0.77083333333333337</v>
+        <v>0.83333333333333337</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">
@@ -2157,22 +2161,22 @@
         <v>115</v>
       </c>
       <c r="B54" t="s">
-        <v>91</v>
+        <v>8</v>
       </c>
       <c r="C54" t="s">
-        <v>23</v>
+        <v>44</v>
       </c>
       <c r="D54" s="2">
-        <v>45867</v>
-      </c>
-      <c r="E54" s="4" t="s">
-        <v>70</v>
+        <v>45854</v>
+      </c>
+      <c r="E54" s="4">
+        <v>14</v>
       </c>
       <c r="F54" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G54" s="3">
-        <v>0.79166666666666663</v>
+        <v>0.89583333333333337</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.35">
@@ -2183,19 +2187,19 @@
         <v>8</v>
       </c>
       <c r="C55" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="D55" s="2">
-        <v>45872</v>
+        <v>45864</v>
       </c>
       <c r="E55" s="4">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F55" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="G55" s="3">
-        <v>0.66666666666666663</v>
+        <v>0.77083333333333337</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.35">
@@ -2203,19 +2207,19 @@
         <v>117</v>
       </c>
       <c r="B56" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="C56" t="s">
-        <v>65</v>
+        <v>23</v>
       </c>
       <c r="D56" s="2">
-        <v>45883</v>
+        <v>45867</v>
       </c>
       <c r="E56" s="4" t="s">
         <v>70</v>
       </c>
       <c r="F56" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G56" s="3">
         <v>0.79166666666666663</v>
@@ -2229,19 +2233,19 @@
         <v>8</v>
       </c>
       <c r="C57" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="D57" s="2">
-        <v>45886</v>
+        <v>45872</v>
       </c>
       <c r="E57" s="4">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F57" t="s">
         <v>13</v>
       </c>
       <c r="G57" s="3">
-        <v>0.85416666666666663</v>
+        <v>0.66666666666666663</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.35">
@@ -2249,22 +2253,22 @@
         <v>119</v>
       </c>
       <c r="B58" t="s">
-        <v>8</v>
+        <v>73</v>
       </c>
       <c r="C58" t="s">
-        <v>23</v>
+        <v>65</v>
       </c>
       <c r="D58" s="2">
-        <v>45899</v>
-      </c>
-      <c r="E58" s="4">
-        <v>22</v>
+        <v>45883</v>
+      </c>
+      <c r="E58" s="4" t="s">
+        <v>70</v>
       </c>
       <c r="F58" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="G58" s="3">
-        <v>0.77083333333333337</v>
+        <v>0.66666666666666663</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.35">
@@ -2272,22 +2276,22 @@
         <v>120</v>
       </c>
       <c r="B59" t="s">
-        <v>91</v>
+        <v>8</v>
       </c>
       <c r="C59" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="D59" s="2">
-        <v>45911</v>
-      </c>
-      <c r="E59" s="4" t="s">
-        <v>71</v>
+        <v>45886</v>
+      </c>
+      <c r="E59" s="4">
+        <v>20</v>
       </c>
       <c r="F59" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G59" s="3">
-        <v>0.89583333333333337</v>
+        <v>0.85416666666666663</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.35">
@@ -2298,128 +2302,128 @@
         <v>8</v>
       </c>
       <c r="C60" t="s">
-        <v>122</v>
+        <v>23</v>
       </c>
       <c r="D60" s="2">
-        <v>45917</v>
+        <v>45899</v>
       </c>
       <c r="E60" s="4">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="F60" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="G60" s="3">
-        <v>0.8125</v>
+        <v>0.77083333333333337</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
+        <v>122</v>
+      </c>
+      <c r="B61" t="s">
+        <v>93</v>
+      </c>
+      <c r="C61" t="s">
+        <v>40</v>
+      </c>
+      <c r="D61" s="2">
+        <v>45911</v>
+      </c>
+      <c r="E61" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="F61" t="s">
+        <v>10</v>
+      </c>
+      <c r="G61" s="3">
+        <v>0.89583333333333337</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
         <v>123</v>
       </c>
-      <c r="B61" t="s">
-        <v>8</v>
-      </c>
-      <c r="C61" t="s">
+      <c r="B62" t="s">
+        <v>8</v>
+      </c>
+      <c r="C62" t="s">
+        <v>124</v>
+      </c>
+      <c r="D62" s="2">
+        <v>45917</v>
+      </c>
+      <c r="E62" s="4">
+        <v>12</v>
+      </c>
+      <c r="F62" t="s">
+        <v>21</v>
+      </c>
+      <c r="G62" s="3">
+        <v>0.8125</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>125</v>
+      </c>
+      <c r="B63" t="s">
+        <v>8</v>
+      </c>
+      <c r="C63" t="s">
         <v>25</v>
       </c>
-      <c r="D61" s="2">
+      <c r="D63" s="2">
         <v>45920</v>
       </c>
-      <c r="E61" s="4">
+      <c r="E63" s="4">
         <v>24</v>
       </c>
-      <c r="F61" t="s">
+      <c r="F63" t="s">
         <v>30</v>
       </c>
-      <c r="G61" s="3">
+      <c r="G63" s="3">
         <v>0.77083333333333337</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A62" s="10" t="s">
-        <v>124</v>
-      </c>
-      <c r="B62" t="s">
-        <v>8</v>
-      </c>
-      <c r="C62" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D62" s="7">
-        <v>45931</v>
-      </c>
-      <c r="E62" s="8">
-        <v>26</v>
-      </c>
-      <c r="F62" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G62" s="9">
-        <v>0.89583333333333337</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A63" s="10" t="s">
-        <v>125</v>
-      </c>
-      <c r="B63" t="s">
-        <v>8</v>
-      </c>
-      <c r="C63" t="s">
-        <v>34</v>
-      </c>
-      <c r="D63" s="2">
-        <v>45945</v>
-      </c>
-      <c r="E63" s="4">
-        <v>28</v>
-      </c>
-      <c r="F63" t="s">
-        <v>21</v>
-      </c>
-      <c r="G63" s="3">
-        <v>0.8125</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="B64" t="s">
-        <v>8</v>
-      </c>
-      <c r="C64" t="s">
-        <v>146</v>
-      </c>
-      <c r="D64" s="2">
-        <v>45956</v>
-      </c>
-      <c r="E64" s="4">
-        <v>30</v>
-      </c>
-      <c r="F64" t="s">
-        <v>13</v>
-      </c>
-      <c r="G64" s="3">
-        <v>0.66666666666666663</v>
+        <v>126</v>
+      </c>
+      <c r="B64" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C64" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D64" s="7">
+        <v>45931</v>
+      </c>
+      <c r="E64" s="8">
+        <v>26</v>
+      </c>
+      <c r="F64" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="G64" s="9">
+        <v>0.89583333333333337</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65" s="10" t="s">
-        <v>131</v>
-      </c>
-      <c r="B65" t="s">
+        <v>127</v>
+      </c>
+      <c r="B65" s="11" t="s">
         <v>8</v>
       </c>
       <c r="C65" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="D65" s="2">
-        <v>45966</v>
+        <v>45945</v>
       </c>
       <c r="E65" s="4">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F65" t="s">
         <v>21</v>
@@ -2432,43 +2436,43 @@
       <c r="A66" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="B66" t="s">
+      <c r="B66" s="11" t="s">
         <v>8</v>
       </c>
       <c r="C66" t="s">
         <v>148</v>
       </c>
       <c r="D66" s="2">
-        <v>45979</v>
+        <v>45956</v>
       </c>
       <c r="E66" s="4">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F66" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="G66" s="3">
-        <v>0.85416666666666663</v>
+        <v>0.66666666666666663</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="B67" t="s">
+      <c r="B67" s="11" t="s">
         <v>8</v>
       </c>
       <c r="C67" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
       <c r="D67" s="2">
-        <v>45983</v>
+        <v>45966</v>
       </c>
       <c r="E67" s="4">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F67" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="G67" s="3">
         <v>0.8125</v>
@@ -2478,326 +2482,372 @@
       <c r="A68" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="B68" t="s">
+      <c r="B68" s="11" t="s">
         <v>8</v>
       </c>
       <c r="C68" t="s">
+        <v>150</v>
+      </c>
+      <c r="D68" s="2">
+        <v>45979</v>
+      </c>
+      <c r="E68" s="4">
+        <v>34</v>
+      </c>
+      <c r="F68" t="s">
+        <v>18</v>
+      </c>
+      <c r="G68" s="3">
+        <v>0.85416666666666663</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A69" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="B69" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C69" t="s">
+        <v>149</v>
+      </c>
+      <c r="D69" s="2">
+        <v>45983</v>
+      </c>
+      <c r="E69" s="4">
+        <v>35</v>
+      </c>
+      <c r="F69" t="s">
+        <v>30</v>
+      </c>
+      <c r="G69" s="3">
+        <v>0.8125</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A70" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="B70" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C70" t="s">
         <v>36</v>
       </c>
-      <c r="D68" s="2">
+      <c r="D70" s="2">
         <v>45998</v>
       </c>
-      <c r="E68" s="4">
+      <c r="E70" s="4">
         <v>38</v>
       </c>
-      <c r="F68" t="s">
+      <c r="F70" t="s">
         <v>13</v>
       </c>
-      <c r="G68" s="3">
+      <c r="G70" s="3">
         <v>0.66666666666666663</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A69" t="s">
-        <v>135</v>
-      </c>
-      <c r="B69" t="s">
-        <v>52</v>
-      </c>
-      <c r="C69" t="s">
-        <v>84</v>
-      </c>
-      <c r="D69" s="2">
-        <v>46043</v>
-      </c>
-      <c r="E69" s="4">
-        <v>3</v>
-      </c>
-      <c r="F69" t="s">
-        <v>21</v>
-      </c>
-      <c r="G69" s="3">
-        <v>0.79166666666666663</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A70" t="s">
-        <v>136</v>
-      </c>
-      <c r="B70" t="s">
-        <v>52</v>
-      </c>
-      <c r="C70" t="s">
-        <v>48</v>
-      </c>
-      <c r="D70" s="2">
-        <v>46046</v>
-      </c>
-      <c r="E70" s="4">
-        <v>4</v>
-      </c>
-      <c r="F70" t="s">
-        <v>30</v>
-      </c>
-      <c r="G70" s="3">
-        <v>0.875</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>137</v>
       </c>
-      <c r="B71" t="s">
-        <v>8</v>
+      <c r="B71" s="11" t="s">
+        <v>52</v>
       </c>
       <c r="C71" t="s">
-        <v>32</v>
+        <v>86</v>
       </c>
       <c r="D71" s="2">
-        <v>46051</v>
+        <v>46043</v>
       </c>
       <c r="E71" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F71" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="G71" s="3">
-        <v>0.89583333333333337</v>
+        <v>0.79166666666666663</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>138</v>
       </c>
-      <c r="B72" t="s">
+      <c r="B72" s="11" t="s">
         <v>52</v>
       </c>
       <c r="C72" t="s">
-        <v>17</v>
+        <v>48</v>
       </c>
       <c r="D72" s="2">
-        <v>46054</v>
+        <v>46046</v>
       </c>
       <c r="E72" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F72" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="G72" s="3">
-        <v>0.85416666666666663</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>139</v>
       </c>
-      <c r="B73" t="s">
-        <v>52</v>
+      <c r="B73" s="11" t="s">
+        <v>8</v>
       </c>
       <c r="C73" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D73" s="2">
-        <v>46068</v>
-      </c>
-      <c r="E73" s="4" t="s">
-        <v>127</v>
+        <v>46051</v>
+      </c>
+      <c r="E73" s="4">
+        <v>1</v>
       </c>
       <c r="F73" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G73" s="3">
-        <v>0.72916666666666663</v>
+        <v>0.89583333333333337</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>140</v>
       </c>
-      <c r="B74" t="s">
-        <v>73</v>
+      <c r="B74" s="11" t="s">
+        <v>52</v>
       </c>
       <c r="C74" t="s">
-        <v>150</v>
+        <v>17</v>
       </c>
       <c r="D74" s="2">
-        <v>46078</v>
-      </c>
-      <c r="E74" s="4" t="s">
-        <v>67</v>
+        <v>46054</v>
+      </c>
+      <c r="E74" s="4">
+        <v>5</v>
       </c>
       <c r="F74" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="G74" s="3">
-        <v>0.89583333333333337</v>
+        <v>0.85416666666666663</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>141</v>
       </c>
-      <c r="B75" t="s">
+      <c r="B75" s="11" t="s">
         <v>52</v>
       </c>
       <c r="C75" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="D75" s="2">
-        <v>46081</v>
+        <v>46068</v>
       </c>
       <c r="E75" s="4" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F75" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="G75" s="3">
-        <v>0.8125</v>
+        <v>0.72916666666666663</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>142</v>
       </c>
-      <c r="B76" t="s">
-        <v>52</v>
+      <c r="B76" s="11" t="s">
+        <v>73</v>
       </c>
       <c r="C76" t="s">
-        <v>48</v>
+        <v>152</v>
       </c>
       <c r="D76" s="2">
-        <v>46088</v>
+        <v>46078</v>
       </c>
       <c r="E76" s="4" t="s">
-        <v>129</v>
+        <v>67</v>
       </c>
       <c r="F76" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="G76" s="3">
-        <v>0.75</v>
+        <v>0.89583333333333337</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>143</v>
       </c>
-      <c r="B77" t="s">
-        <v>73</v>
+      <c r="B77" s="11" t="s">
+        <v>52</v>
       </c>
       <c r="C77" t="s">
-        <v>149</v>
+        <v>51</v>
       </c>
       <c r="D77" s="2">
-        <v>46091</v>
+        <v>46081</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="F77" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="G77" s="3">
-        <v>0.89583333333333337</v>
+        <v>0.8125</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>144</v>
       </c>
-      <c r="B78" t="s">
-        <v>8</v>
+      <c r="B78" s="11" t="s">
+        <v>52</v>
       </c>
       <c r="C78" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="D78" s="2">
-        <v>46095</v>
-      </c>
-      <c r="E78" s="4">
-        <v>6</v>
+        <v>46088</v>
+      </c>
+      <c r="E78" s="4" t="s">
+        <v>131</v>
       </c>
       <c r="F78" t="s">
         <v>30</v>
       </c>
       <c r="G78" s="3">
-        <v>0.85416666666666663</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>145</v>
       </c>
-      <c r="B79" t="s">
-        <v>8</v>
+      <c r="B79" s="11" t="s">
+        <v>73</v>
       </c>
       <c r="C79" t="s">
-        <v>122</v>
+        <v>151</v>
       </c>
       <c r="D79" s="2">
-        <v>46113</v>
-      </c>
-      <c r="E79" s="4">
-        <v>9</v>
+        <v>46091</v>
+      </c>
+      <c r="E79" s="4" t="s">
+        <v>128</v>
       </c>
       <c r="F79" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G79" s="3">
-        <v>0.8125</v>
+        <v>0.89583333333333337</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>154</v>
-      </c>
-      <c r="B80" t="s">
-        <v>151</v>
+        <v>146</v>
+      </c>
+      <c r="B80" s="11" t="s">
+        <v>8</v>
       </c>
       <c r="C80" t="s">
-        <v>153</v>
+        <v>34</v>
       </c>
       <c r="D80" s="2">
-        <v>46121</v>
-      </c>
-      <c r="E80" s="4" t="s">
-        <v>69</v>
+        <v>46095</v>
+      </c>
+      <c r="E80" s="4">
+        <v>6</v>
       </c>
       <c r="F80" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="G80" s="3">
-        <v>0.79166666666666663</v>
+        <v>0.85416666666666663</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
+        <v>147</v>
+      </c>
+      <c r="B81" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C81" t="s">
+        <v>124</v>
+      </c>
+      <c r="D81" s="2">
+        <v>46113</v>
+      </c>
+      <c r="E81" s="4">
+        <v>9</v>
+      </c>
+      <c r="F81" t="s">
+        <v>21</v>
+      </c>
+      <c r="G81" s="3">
+        <v>0.8125</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
+        <v>156</v>
+      </c>
+      <c r="B82" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="C82" t="s">
         <v>155</v>
       </c>
-      <c r="B81" t="s">
-        <v>8</v>
-      </c>
-      <c r="C81" t="s">
-        <v>152</v>
-      </c>
-      <c r="D81" s="2">
+      <c r="D82" s="2">
+        <v>46121</v>
+      </c>
+      <c r="E82" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="F82" t="s">
+        <v>10</v>
+      </c>
+      <c r="G82" s="3">
+        <v>0.79166666666666663</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>157</v>
+      </c>
+      <c r="B83" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C83" t="s">
+        <v>154</v>
+      </c>
+      <c r="D83" s="2">
         <v>46124</v>
       </c>
-      <c r="E81" s="4">
+      <c r="E83" s="4">
         <v>11</v>
       </c>
-      <c r="F81" t="s">
+      <c r="F83" t="s">
         <v>13</v>
       </c>
-      <c r="G81" s="3">
+      <c r="G83" s="3">
         <v>0.66666666666666663</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G81" xr:uid="{2921BBCD-6E27-463C-B492-0BF065778598}"/>
+  <autoFilter ref="A1:G64" xr:uid="{2921BBCD-6E27-463C-B492-0BF065778598}"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
data: atualiza xlsx e regenera data.js + placares.js
Novos xlsx: dPartidas, dPlacares, dTimes, dTorcedores, fFacial, fIngressos.
data.js: 87 partidas, 4294 ingressos, faturamento total R$52.5M.
placares.js: 182 jogos até 20/05/2026.
</commit_message>
<xml_diff>
--- a/dPartidas.xlsx
+++ b/dPartidas.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="EstaPastaDeTrabalho" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://safbotafogo-my.sharepoint.com/personal/pedro_arruda_safbfr_com_br/Documents/Área de Trabalho/dash-ticket/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="477" documentId="8_{E25D5179-CBFE-42C3-9E8D-799BA19C3FB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15D5C576-7611-44B6-AFD0-EE56B32D2144}"/>
+  <xr:revisionPtr revIDLastSave="525" documentId="8_{E25D5179-CBFE-42C3-9E8D-799BA19C3FB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08B0B72D-C7EF-404B-A12F-898B84764E4E}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E1B40A1D-D5F1-4DC5-B00D-B969B491F639}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Planilha3" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha3!$A$1:$G$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha3!$A$1:$G$88</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="167">
   <si>
     <t>ID_PARTIDA</t>
   </si>
@@ -513,6 +513,33 @@
   </si>
   <si>
     <t>2026.04.12-CAMBR2-11</t>
+  </si>
+  <si>
+    <t>29CHBRSC</t>
+  </si>
+  <si>
+    <t>35REBRPA</t>
+  </si>
+  <si>
+    <t>124IPBOSU</t>
+  </si>
+  <si>
+    <t>5° Fase</t>
+  </si>
+  <si>
+    <t>2026.04.21-CAMCO3-5° Fase</t>
+  </si>
+  <si>
+    <t>2026.04.28-CAMSU6-FG</t>
+  </si>
+  <si>
+    <t>2026.05.02-CAMBR2-14</t>
+  </si>
+  <si>
+    <t>2026.05.06-CAMSU6-FG</t>
+  </si>
+  <si>
+    <t>2026.05.17-CAMBR2-16</t>
   </si>
 </sst>
 </file>
@@ -574,7 +601,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -592,7 +619,6 @@
     </xf>
     <xf numFmtId="20" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -928,7 +954,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2921BBCD-6E27-463C-B492-0BF065778598}">
   <sheetPr codeName="Planilha1"/>
-  <dimension ref="A1:G83"/>
+  <dimension ref="A1:G88"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.81640625" bestFit="1" customWidth="1"/>
@@ -1985,8 +2011,8 @@
       <c r="D46" s="2">
         <v>45755</v>
       </c>
-      <c r="E46" s="4">
-        <v>2</v>
+      <c r="E46" s="4" t="s">
+        <v>69</v>
       </c>
       <c r="F46" t="s">
         <v>18</v>
@@ -2100,8 +2126,8 @@
       <c r="D51" s="2">
         <v>45791</v>
       </c>
-      <c r="E51" s="4">
-        <v>5</v>
+      <c r="E51" s="4" t="s">
+        <v>69</v>
       </c>
       <c r="F51" t="s">
         <v>21</v>
@@ -2123,8 +2149,8 @@
       <c r="D52" s="2">
         <v>45804</v>
       </c>
-      <c r="E52" s="4">
-        <v>6</v>
+      <c r="E52" s="4" t="s">
+        <v>69</v>
       </c>
       <c r="F52" t="s">
         <v>18</v>
@@ -2390,7 +2416,7 @@
       <c r="A64" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="B64" s="11" t="s">
+      <c r="B64" t="s">
         <v>8</v>
       </c>
       <c r="C64" s="5" t="s">
@@ -2413,7 +2439,7 @@
       <c r="A65" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="B65" s="11" t="s">
+      <c r="B65" t="s">
         <v>8</v>
       </c>
       <c r="C65" t="s">
@@ -2436,7 +2462,7 @@
       <c r="A66" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="B66" s="11" t="s">
+      <c r="B66" t="s">
         <v>8</v>
       </c>
       <c r="C66" t="s">
@@ -2459,7 +2485,7 @@
       <c r="A67" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="B67" s="11" t="s">
+      <c r="B67" t="s">
         <v>8</v>
       </c>
       <c r="C67" t="s">
@@ -2482,7 +2508,7 @@
       <c r="A68" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="B68" s="11" t="s">
+      <c r="B68" t="s">
         <v>8</v>
       </c>
       <c r="C68" t="s">
@@ -2505,7 +2531,7 @@
       <c r="A69" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="B69" s="11" t="s">
+      <c r="B69" t="s">
         <v>8</v>
       </c>
       <c r="C69" t="s">
@@ -2528,7 +2554,7 @@
       <c r="A70" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="B70" s="11" t="s">
+      <c r="B70" t="s">
         <v>8</v>
       </c>
       <c r="C70" t="s">
@@ -2551,7 +2577,7 @@
       <c r="A71" t="s">
         <v>137</v>
       </c>
-      <c r="B71" s="11" t="s">
+      <c r="B71" t="s">
         <v>52</v>
       </c>
       <c r="C71" t="s">
@@ -2574,7 +2600,7 @@
       <c r="A72" t="s">
         <v>138</v>
       </c>
-      <c r="B72" s="11" t="s">
+      <c r="B72" t="s">
         <v>52</v>
       </c>
       <c r="C72" t="s">
@@ -2597,7 +2623,7 @@
       <c r="A73" t="s">
         <v>139</v>
       </c>
-      <c r="B73" s="11" t="s">
+      <c r="B73" t="s">
         <v>8</v>
       </c>
       <c r="C73" t="s">
@@ -2620,7 +2646,7 @@
       <c r="A74" t="s">
         <v>140</v>
       </c>
-      <c r="B74" s="11" t="s">
+      <c r="B74" t="s">
         <v>52</v>
       </c>
       <c r="C74" t="s">
@@ -2643,7 +2669,7 @@
       <c r="A75" t="s">
         <v>141</v>
       </c>
-      <c r="B75" s="11" t="s">
+      <c r="B75" t="s">
         <v>52</v>
       </c>
       <c r="C75" t="s">
@@ -2666,7 +2692,7 @@
       <c r="A76" t="s">
         <v>142</v>
       </c>
-      <c r="B76" s="11" t="s">
+      <c r="B76" t="s">
         <v>73</v>
       </c>
       <c r="C76" t="s">
@@ -2689,7 +2715,7 @@
       <c r="A77" t="s">
         <v>143</v>
       </c>
-      <c r="B77" s="11" t="s">
+      <c r="B77" t="s">
         <v>52</v>
       </c>
       <c r="C77" t="s">
@@ -2712,7 +2738,7 @@
       <c r="A78" t="s">
         <v>144</v>
       </c>
-      <c r="B78" s="11" t="s">
+      <c r="B78" t="s">
         <v>52</v>
       </c>
       <c r="C78" t="s">
@@ -2735,7 +2761,7 @@
       <c r="A79" t="s">
         <v>145</v>
       </c>
-      <c r="B79" s="11" t="s">
+      <c r="B79" t="s">
         <v>73</v>
       </c>
       <c r="C79" t="s">
@@ -2758,7 +2784,7 @@
       <c r="A80" t="s">
         <v>146</v>
       </c>
-      <c r="B80" s="11" t="s">
+      <c r="B80" t="s">
         <v>8</v>
       </c>
       <c r="C80" t="s">
@@ -2781,7 +2807,7 @@
       <c r="A81" t="s">
         <v>147</v>
       </c>
-      <c r="B81" s="11" t="s">
+      <c r="B81" t="s">
         <v>8</v>
       </c>
       <c r="C81" t="s">
@@ -2804,7 +2830,7 @@
       <c r="A82" t="s">
         <v>156</v>
       </c>
-      <c r="B82" s="11" t="s">
+      <c r="B82" t="s">
         <v>153</v>
       </c>
       <c r="C82" t="s">
@@ -2827,7 +2853,7 @@
       <c r="A83" t="s">
         <v>157</v>
       </c>
-      <c r="B83" s="11" t="s">
+      <c r="B83" t="s">
         <v>8</v>
       </c>
       <c r="C83" t="s">
@@ -2846,8 +2872,123 @@
         <v>0.66666666666666663</v>
       </c>
     </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
+        <v>162</v>
+      </c>
+      <c r="B84" t="s">
+        <v>93</v>
+      </c>
+      <c r="C84" t="s">
+        <v>158</v>
+      </c>
+      <c r="D84" s="2">
+        <v>46133</v>
+      </c>
+      <c r="E84" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="F84" t="s">
+        <v>18</v>
+      </c>
+      <c r="G84" s="3">
+        <v>0.70833333333333337</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>163</v>
+      </c>
+      <c r="B85" t="s">
+        <v>153</v>
+      </c>
+      <c r="C85" t="s">
+        <v>160</v>
+      </c>
+      <c r="D85" s="2">
+        <v>46140</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="F85" t="s">
+        <v>18</v>
+      </c>
+      <c r="G85" s="3">
+        <v>0.79166666666666663</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
+        <v>164</v>
+      </c>
+      <c r="B86" t="s">
+        <v>8</v>
+      </c>
+      <c r="C86" t="s">
+        <v>159</v>
+      </c>
+      <c r="D86" s="2">
+        <v>46144</v>
+      </c>
+      <c r="E86" s="4">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>30</v>
+      </c>
+      <c r="G86" s="3">
+        <v>0.66666666666666663</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
+        <v>165</v>
+      </c>
+      <c r="B87" t="s">
+        <v>153</v>
+      </c>
+      <c r="C87" t="s">
+        <v>103</v>
+      </c>
+      <c r="D87" s="2">
+        <v>46148</v>
+      </c>
+      <c r="E87" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="F87" t="s">
+        <v>21</v>
+      </c>
+      <c r="G87" s="3">
+        <v>0.89583333333333337</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
+        <v>166</v>
+      </c>
+      <c r="B88" t="s">
+        <v>8</v>
+      </c>
+      <c r="C88" t="s">
+        <v>38</v>
+      </c>
+      <c r="D88" s="2">
+        <v>46159</v>
+      </c>
+      <c r="E88" s="4">
+        <v>16</v>
+      </c>
+      <c r="F88" t="s">
+        <v>13</v>
+      </c>
+      <c r="G88" s="3">
+        <v>0.66666666666666663</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G64" xr:uid="{2921BBCD-6E27-463C-B492-0BF065778598}"/>
+  <autoFilter ref="A1:G88" xr:uid="{2921BBCD-6E27-463C-B492-0BF065778598}"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>